<commit_message>
Add 0714_Learning Materials downloads card and hide official content tab for course-0vvk06
</commit_message>
<xml_diff>
--- a/courses/course-0vvk06/prep/downloads/實作提示_20260714.xlsx
+++ b/courses/course-0vvk06/prep/downloads/實作提示_20260714.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ting_hsia\.gemini\antigravity\scratch\learning-hub\courses\course-0vvk06\prep\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7A6E34-09B2-402D-BC1E-8026D8F1FEBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FBF34E9-AAFF-49BC-8277-5937A70A2206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1079,6 +1079,55 @@
     <t>-</t>
   </si>
   <si>
+    <t>第三題：網站價格監控</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>利用 Playwright 進行自動網頁爬取，能定時監控網站商品的價格波動，並在售價低於期望值時自動提醒與匯出歷史報表。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我想做出一個 Windows 電腦上運行的桌面應用程式，用來幫我監控 ASUS 官網的筆電價格。
+請幫我用最簡單、穩定的方式寫出完整程式碼，並告訴我如何安裝與執行。
+我的具體需求如下：
+1. 監控的網頁：
+   - 請去這個公開網頁爬取資料：https://www.asus.com/tw/laptops/for-home/all-series/filter?Spec=126640
+     （這個網頁已經篩選了「有庫存」的筆電）。
+   - 因為是公開網站，不需要登入，也不需要 VPN。
+     網頁是動態載入的，請確保程式能自動滾動網頁載入所有商品後再擷取資料。
+   - 請幫我記錄每一台筆電的「品名」、「最新售價」和「更新時間」。
+     如果同一台筆電顯示兩個價格，請忽略有刪除線的原價，只抓實際售價。
+2. 軟體畫面與功能（請使用繁體中文、簡約的藍白配色）：
+   - 左邊面板：讓我輸入「商品關鍵字」與「我的期望最高價格」，
+     並有一個清單顯示我正在監控哪些規則。
+   - 右邊面板：顯示兩個分頁：
+     - 第一個分頁「目前最新價格」：用卡片方式列出所有抓到的筆電。
+     - 第二個分頁「歷史更新紀錄」：列出所有爬取時間點。
+   - 價格變化提示：在最新價格的卡片上，
+     如果這台筆電這次的售價比上次低，請在價格旁用綠色顯示「(↓ 降價金額)」；
+     如果變貴了，用紅色顯示「(↑ 漲價金額)」。
+   - 細項歷史與下載：當我點選卡片上的「查看歷史」按鈕時，
+     請彈出一個小視窗，用表格顯示這台筆電所有歷史價格與更新時間，
+     並在視窗中提供一個「下載此品項歷史 (CSV)」的按鈕。
+   - 匯出全部：在主畫面提供一個按鈕，讓我一鍵下載目前資料庫所有的歷史價格紀錄為 CSV 檔案。
+3. 背景監控與警報：
+   - 在主畫面下方提供「立即手動更新價格」按鈕，
+     以及「自動定期監控」開關與間隔時間（如 15 分鐘、1 小時）。
+   - 當爬取到的售價低於我設定的「期望價格」時，
+     請自動彈出 Windows 系統的通知訊息（通知中心氣球提示）來提醒我。
+4. 啟動與部署方式（請嚴格遵守以下限制，以防範 Windows 環境常見的閃退與多餘視窗問題）：
+   a. 請只生成以下兩個啟動檔案，不要建立其他額外的 .bat 檔案：
+      - run_app.bat：直接執行應用程式（前台開啟，方便調試或顯示畫面）。
+      - 啟動價格監控.vbs：利用 pythonw.exe 在背景無視窗執行（後台靜默開啟）。
+   b. 所有的套件偵測與安裝邏輯必須寫在 Python 程式碼中，不可寫在批次檔中：
+      - 程式啟動時，應自動偵測爬蟲套件（如 playwright 或 selenium）、圖形介面套件（customtkinter）、與系統通知套件（plyer）是否已安裝。
+      - 若未安裝，自動呼叫 `pip install` 進行下載安裝。如果使用的是 playwright，安裝完套件後需自動執行 `playwright install chromium`。
+   c. 路徑與環境穩定性：
+      - 啟動時請使用 `sys.executable` 取得當前環境 python.exe 的絕對路徑，並由此推導出 pythonw.exe 的路徑，不可依賴系統 PATH（因為 pythonw.exe 通常不在 PATH 中）。
+      - 執行 `啟動價格監控.vbs` 後，黑色的 CMD 視窗必須瞬間關閉（或根本不出現），而主程式能順利在背景執行且不會閃退。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>我想要在網頁上新增一個「批次檔案匯入」的功能，可以支援上傳信用卡對帳單的 PDF 檔或圖片檔（JPG, PNG），並自動抓取裡面的交易明細，具體需求如下：
 1. 檔案讀取方式：
    - 如果是圖片檔，請利用離線 OCR 引擎（文字辨識）來辨識圖中的文字。
@@ -1093,34 +1142,6 @@
      - 中間顯示一個簡約的 7 欄表格（刷卡日期、帳單起息日、明細、金額、地區、分類、操作），使用者可以直接在表格內手動修改，或者點操作欄的垃圾桶圖示刪除該筆錯誤資料。
      - 視窗底部除了「取消」與「確認匯入資料庫」外，必須有「捨棄此檔案」按鈕，讓我可以跳過或刪除整張解析失敗的檔案。
 請以藍白簡約、專業質感的網頁風格來設計此介面，謝謝！</t>
-  </si>
-  <si>
-    <t>第三題：網站價格監控</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>利用 Playwright 進行自動網頁爬取，能定時監控網站商品的價格波動，並在售價低於期望值時自動提醒與匯出歷史報表。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>我想做出一個 Windows 電腦上運行的桌面應用程式，用來幫我監控 ASUS 官網的筆電價格。請幫我用最簡單、穩定的方式寫出完整程式碼，並告訴我如何安裝與執行。
-我的具體需求如下：
-1. 監控的網頁：
-   - 請去這個公開網頁爬取資料：https://www.asus.com/tw/laptops/for-home/all-series/filter?Spec=126640 （這個網頁已經篩選了「有庫存」的筆電）。
-   - 因為是公開網站，不需要登入，也不需要 VPN。網頁是動態載入的，請確保程式能自動滾動網頁載入所有商品後再擷取資料。
-   - 請幫我記錄每一台筆電的「品名」、「最新售價」和「更新時間」。如果同一台筆電顯示兩個價格，請忽略有刪除線的原價，只抓實際售價。
-2. 軟體畫面與功能（請使用繁體中文、簡約的藍白配色）：
-   - 左邊面板：讓我輸入「商品關鍵字」與「我的期望最高價格」，並有一個清單顯示我正在監控哪些規則。
-   - 右邊面板：顯示兩個分頁，第一個分頁是「目前最新價格」，用卡片方式列出所有抓到的筆電；第二個分頁是「歷史更新紀錄」，列出所有爬取時間點。
-   - 價格變化提示：在最新價格的卡片上，如果這台筆電這次的售價比上次低，請在價格旁用綠色顯示「(↓ 降價金額)」；如果變貴了，用紅色顯示「(↑ 漲價金額)」。
-   - 細項歷史與下載：當我點選卡片上的「查看歷史」按鈕時，請彈出一個小視窗，用表格顯示這台筆電所有歷史價格與更新時間，並在視窗中提供一個「下載此品項歷史 (CSV)」的按鈕。
-   - 匯出全部：在主畫面提供一個按鈕，讓我一鍵下載目前資料庫所有的歷史價格紀錄為 CSV 檔案。
-3. 背景監控與警報：
-   - 在主畫面下方提供「立即手動更新價格」按鈕，以及「自動定期監控」開關與間隔時間（如 15 分鐘、1 小時）。
-   - 當爬取到的售價低於我設定的「期望價格」時，請自動彈出 Windows 系統的通知訊息（通知中心氣球提示）來提醒我。
-4. 啟動與封包方式：
-   - 我希望可以一鍵啟動它。請幫我寫一個 VBS 啟動腳本或批次檔，讓我雙擊後，程式能默默在電腦背景開啟並跑出畫面，不要殘留一個黑色的 CMD 命令提示字元視窗。
-   - 所有的程式碼、資料庫和啟動檔請都包在同一個資料夾中，不要在桌面產生捷徑，方便我以後整包複製分享給別人。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1763,21 +1784,21 @@
         <v>42</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>45</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update course hints from Excel and implement server-side path traversal and XSS security mitigations
</commit_message>
<xml_diff>
--- a/courses/course-0vvk06/prep/downloads/實作提示_20260714.xlsx
+++ b/courses/course-0vvk06/prep/downloads/實作提示_20260714.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ting_hsia\.gemini\antigravity\scratch\learning-hub\courses\course-0vvk06\prep\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FBF34E9-AAFF-49BC-8277-5937A70A2206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5941AB35-163F-4F78-ADEA-3FF5DD108224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1087,47 +1087,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>我想做出一個 Windows 電腦上運行的桌面應用程式，用來幫我監控 ASUS 官網的筆電價格。
-請幫我用最簡單、穩定的方式寫出完整程式碼，並告訴我如何安裝與執行。
-我的具體需求如下：
-1. 監控的網頁：
-   - 請去這個公開網頁爬取資料：https://www.asus.com/tw/laptops/for-home/all-series/filter?Spec=126640
-     （這個網頁已經篩選了「有庫存」的筆電）。
-   - 因為是公開網站，不需要登入，也不需要 VPN。
-     網頁是動態載入的，請確保程式能自動滾動網頁載入所有商品後再擷取資料。
-   - 請幫我記錄每一台筆電的「品名」、「最新售價」和「更新時間」。
-     如果同一台筆電顯示兩個價格，請忽略有刪除線的原價，只抓實際售價。
-2. 軟體畫面與功能（請使用繁體中文、簡約的藍白配色）：
-   - 左邊面板：讓我輸入「商品關鍵字」與「我的期望最高價格」，
-     並有一個清單顯示我正在監控哪些規則。
-   - 右邊面板：顯示兩個分頁：
-     - 第一個分頁「目前最新價格」：用卡片方式列出所有抓到的筆電。
-     - 第二個分頁「歷史更新紀錄」：列出所有爬取時間點。
-   - 價格變化提示：在最新價格的卡片上，
-     如果這台筆電這次的售價比上次低，請在價格旁用綠色顯示「(↓ 降價金額)」；
-     如果變貴了，用紅色顯示「(↑ 漲價金額)」。
-   - 細項歷史與下載：當我點選卡片上的「查看歷史」按鈕時，
-     請彈出一個小視窗，用表格顯示這台筆電所有歷史價格與更新時間，
-     並在視窗中提供一個「下載此品項歷史 (CSV)」的按鈕。
-   - 匯出全部：在主畫面提供一個按鈕，讓我一鍵下載目前資料庫所有的歷史價格紀錄為 CSV 檔案。
-3. 背景監控與警報：
-   - 在主畫面下方提供「立即手動更新價格」按鈕，
-     以及「自動定期監控」開關與間隔時間（如 15 分鐘、1 小時）。
-   - 當爬取到的售價低於我設定的「期望價格」時，
-     請自動彈出 Windows 系統的通知訊息（通知中心氣球提示）來提醒我。
-4. 啟動與部署方式（請嚴格遵守以下限制，以防範 Windows 環境常見的閃退與多餘視窗問題）：
-   a. 請只生成以下兩個啟動檔案，不要建立其他額外的 .bat 檔案：
-      - run_app.bat：直接執行應用程式（前台開啟，方便調試或顯示畫面）。
-      - 啟動價格監控.vbs：利用 pythonw.exe 在背景無視窗執行（後台靜默開啟）。
-   b. 所有的套件偵測與安裝邏輯必須寫在 Python 程式碼中，不可寫在批次檔中：
-      - 程式啟動時，應自動偵測爬蟲套件（如 playwright 或 selenium）、圖形介面套件（customtkinter）、與系統通知套件（plyer）是否已安裝。
-      - 若未安裝，自動呼叫 `pip install` 進行下載安裝。如果使用的是 playwright，安裝完套件後需自動執行 `playwright install chromium`。
-   c. 路徑與環境穩定性：
-      - 啟動時請使用 `sys.executable` 取得當前環境 python.exe 的絕對路徑，並由此推導出 pythonw.exe 的路徑，不可依賴系統 PATH（因為 pythonw.exe 通常不在 PATH 中）。
-      - 執行 `啟動價格監控.vbs` 後，黑色的 CMD 視窗必須瞬間關閉（或根本不出現），而主程式能順利在背景執行且不會閃退。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>我想要在網頁上新增一個「批次檔案匯入」的功能，可以支援上傳信用卡對帳單的 PDF 檔或圖片檔（JPG, PNG），並自動抓取裡面的交易明細，具體需求如下：
 1. 檔案讀取方式：
    - 如果是圖片檔，請利用離線 OCR 引擎（文字辨識）來辨識圖中的文字。
@@ -1142,6 +1101,42 @@
      - 中間顯示一個簡約的 7 欄表格（刷卡日期、帳單起息日、明細、金額、地區、分類、操作），使用者可以直接在表格內手動修改，或者點操作欄的垃圾桶圖示刪除該筆錯誤資料。
      - 視窗底部除了「取消」與「確認匯入資料庫」外，必須有「捨棄此檔案」按鈕，讓我可以跳過或刪除整張解析失敗的檔案。
 請以藍白簡約、專業質感的網頁風格來設計此介面，謝謝！</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>請幫我製作一個 Windows 電腦上運行的原生桌面應用程式，用來監控 ASUS 官網的筆電價格，並在降價至期望價格以下時發送系統通知。請使用 Python 與 SQLite 開發，並以最簡潔、極致穩定的架構寫出完整程式碼，並告訴我如何執行。
+1. 系統架構與穩定性要求 (關鍵核心)
+- 行程分離設計：為避免 Playwright 瀏覽器自動化在非同步/多執行緒（如 Tkinter 背景執行緒或 pythonw.exe）下運行發生 Event Loop 死鎖或崩潰，必須將系統拆分為四個獨立的檔案：
+  1. database.py：負責 SQLite 資料庫 (price_monitor.db) 的初始化與所有增刪查改操作（包含警報規則、價格歷史與已發送通知紀錄）。資料庫路徑必須基於腳本的絕對路徑，以確保工作排程器執行時能正確定位。
+  2. scraper.py：獨立的爬蟲行程。由 main.py 透過 subprocess.run 啟動。使用 Playwright 無頭 Chromium 模擬滾動到底部以加載所有商品。爬取結果必須以 json.dumps(..., ensure_ascii=True) 序列化為 ASCII-escaped JSON 格式輸出至 stdout，過程日誌與錯誤則輸出至 stderr，以防止 Windows 控制台（如 CP950）在重導向 stdout 時因讀取到不相容字元而崩潰。
+  3. main.py：負責桌面 GUI 介面的展示與定時輪詢核心，支援獨立執行緒啟動 scraper.py，且支援 --headless 命令行參數。
+     - 隱藏執行：呼叫 scraper.py 時，若目前以 pythonw.exe 執行，必須自動替換為 python.exe（確保 Playwright 正常啟動），並透過設定 Windows startupinfo.wShowWindow = 0 (SW_HIDE) 旗標，將彈出的爬蟲 CMD 黑視窗完全隱藏。
+  4. run_app.bat：一鍵啟動批處理檔。用來雙擊直接執行 python main.py。若發生執行出錯，視窗應保持開啟並提示使用者安裝依賴（pip install customtkinter playwright）。
+- 無介面排程支援 (Headless Mode)：
+  main.py 必須支援 --headless 命令行參數（即執行 python main.py --headless）。在此模式下，程式不啟動 GUI 介面，而是直接在背景執行一次爬蟲調用、寫入資料庫、比對期望價規則、觸發系統通知後即自動關閉，以利配合 Windows 工作排程器定時執行。
+- 資料庫：在同目錄下使用 SQLite (price_monitor.db) 儲存規則、價格歷史，以及 notifications_sent 發送紀錄。
+2. 介面美感要求 (SaaS 科技藍雙色調儀表板)
+請使用 CustomTkinter (customtkinter) 庫進行扁平化現代設計（預設設為 AppearanceMode: light, ColorTheme: blue）：
+- 左側邊欄 (深色主題 - #0f172a)：
+  品牌名稱區、新增規則區、規則列表、監控開關與手動更新按鈕。
+  輸入框改為深色扁平設計 (fg_color="#1e293b", border_color="#334155")。由於 CTkEntry 不支援建構子內直接傳入 focused_border_color，必須手動綁定 &lt;FocusIn&gt; 與 &lt;FocusOut&gt; 事件，在 Focused 時將 border color 設為科技藍 #3b82f6 實現動態高亮。
+  規則列表的卡片使用 #1e293b 作為背景並包含紅色 × 的刪除按鈕。使用平面 Frame 與細線作為區塊分隔，不使用傳統的凹凸 LabelFrame 框。
+- 右側主面板 (淺色主題 - #f8fafc)：
+  頂部配置軟藍色 (#f1f5f9) 圓角膠囊狀態列，帶有綠色連線指示燈 ● （於自動更新/手動更新時變更顏色與文字狀態）與最後更新時間。
+  顯示兩個分頁：「目前最新價格」與「歷史更新紀錄」（以 CTkTabview 呈現）。
+- 響應式垂直卡片 (Latest Prices Tab)：
+  每台筆電為一個純白 (#ffffff) 懸浮卡片，具備灰色細框。透過遞迴綁定 &lt;Enter&gt; 與 &lt;Leave&gt; 事件（跳過 CTkButton），在滑鼠移入時將邊框顏色改為科技藍，移出時復原。
+  版面必須為垂直堆疊 (Vertical Stack)：上層為品名（Wraplength 設定為 700 左右，隨視窗縮小自動換行）；下層為左右對齊（左側為價格與漲跌幅度膠囊 Badge，右側為「查看歷史」按鈕）。這可確保縮小視窗時，按鈕與文字絕對不被遮擋或重疊。
+- 價格變化提示：比上次降價用綠色標章顯示 (↓ 降價金額，背景 #dcfce7，字體 #15803d)；漲價用紅色標章顯示 (↑ 漲價金額，背景 #fee2e2，字體 #b91c1c)；無變動用灰色顯示 (無變動)。
+- 斑馬紋數據表格 (Treeview)：
+  更新紀錄表格與單品歷史彈窗，使用標準 ttk.Treeview 並設定 style.theme_use('clam') 以便配置自訂色彩。將背景設為 #ffffff，奇數行設置標籤 odd 背景為 #f8fafc。配合使用 CTkScrollbar 替代傳統 Tkinter 滾動條以符合 CustomTkinter 設計語言，且移除 Treeview 預設的厚重外邊框。
+3. 功能細節要求
+- 爬蟲邏輯：爬取 https://www.asus.com/tw/laptops/for-home/all-series/filter?Spec=126640。啟動 Playwright 無頭 Chromium，模擬滾動到底部以加載所有商品（滾動 6 次，每次間隔 1.5 秒）。
+  - Selectors：商品卡片使用 div[class*="ProductCardNormalGrid__productCardContainer"]；商品名稱使用 a[class*="headingRow"] h2 或 a[class*="headingRow"]；連結使用 a[class*="headingRow"] 的 href 屬性；當前實售價使用 div[class*="ProductCardNormalGrid__price__"]（過濾掉含有 regularPrice 類名的刪除線原價）。
+- 警報通知：新增規則時，模糊比對商品品名（不區分大小寫）。當 當前實售價 &lt;= 期望價 時，若該商品在資料庫中為初次符合或價格有變動，調用 PowerShell BalloonTip 彈出 Windows 系統通知，不重複發送相同價格的通知。
+- 歷史彈窗與匯出：
+  點選卡片「查看歷史」彈出 CTkToplevel 模態小視窗，用表格列出此商品所有歷史價格。
+  支援「匯出全體歷史 (CSV)」與單品「下載歷史 (CSV)」。匯出 CSV 時，開啟檔案必須使用 Python 的 utf-8-sig 編碼寫入（即自動添加 UTF-8 BOM \ufeff 標記），以防止 Windows 使用者雙擊 Excel 直接開啟時中文內容產生亂碼。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1784,7 +1779,7 @@
         <v>42</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1798,7 +1793,7 @@
         <v>42</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Vibe Coding topics and sync latest Excel contents to data.json
</commit_message>
<xml_diff>
--- a/courses/course-0vvk06/prep/downloads/實作提示_20260714.xlsx
+++ b/courses/course-0vvk06/prep/downloads/實作提示_20260714.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ting_hsia\.gemini\antigravity\scratch\learning-hub\courses\course-0vvk06\prep\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5941AB35-163F-4F78-ADEA-3FF5DD108224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89EF800-58DA-4EA2-9A29-000A35049E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -856,9 +856,6 @@
     <t>Agy提示詞</t>
   </si>
   <si>
-    <t>第一題：信用卡記帳管理系統</t>
-  </si>
-  <si>
     <t>透過上述VBA實作彙整，進行記帳系統的軟體開發</t>
   </si>
   <si>
@@ -1028,6 +1025,103 @@
 End Sub</t>
   </si>
   <si>
+    <t>PDF解析是提取原生向量文字物件，並透過演算法進行結構重組；而圖片辨識則是藉由光學字元辨識(OCR)進行特徵提取與字元重建。</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>利用 Playwright 進行自動網頁爬取，能定時監控網站商品的價格波動，並在售價低於期望值時自動提醒與匯出歷史報表。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我想要在網頁上新增一個「批次檔案匯入」的功能，可以支援上傳信用卡對帳單的 PDF 檔或圖片檔（JPG, PNG），並自動抓取裡面的交易明細，具體需求如下：
+1. 檔案讀取方式：
+   - 如果是圖片檔，請利用離線 OCR 引擎（文字辨識）來辨識圖中的文字。
+   - 如果是 PDF 檔，因為裡面本來就有文字定義，請直接用 PDF 的文字提取方式讀取，不需要用 OCR，並請確保能把同一橫排的文字（日期、明細、金額）正確拼湊在一起，避免行與行之間對不齊。
+2. 資料抓取與雜訊過濾：
+   - 幫我從檔案內容中抓出每筆刷卡的：消費日期、消費明細（如果有英文字中間多餘的空格請幫我刪除）、消費金額、消費地區。
+   - 排除雜訊：帳單內常會出現「信用卡卡號、最低應繳金額、本期應繳總金額、結帳日、繳款截止日、持卡人姓名」等數字，請幫我寫規則過濾掉，不要把它們誤認成消費金額。
+3. 交易明細確認視窗（使用者審核介面）：
+   - 解析完成後，請彈出一個名為「交易明細確認」的簡約視窗，讓我們逐一確認每個檔案的內容：
+     - 視窗頂部要有一個「檔案審核進度條」（例如：第 1 / 3 個檔案），讓我知道還有幾張要確認。
+     - 頂部可以設定「此檔案所屬銀行」，並會自動偵測帳單文字來預填銀行名稱。
+     - 中間顯示一個簡約的 7 欄表格（刷卡日期、帳單起息日、明細、金額、地區、分類、操作），使用者可以直接在表格內手動修改，或者點操作欄的垃圾桶圖示刪除該筆錯誤資料。
+     - 視窗底部除了「取消」與「確認匯入資料庫」外，必須有「捨棄此檔案」按鈕，讓我可以跳過或刪除整張解析失敗的檔案。
+請以藍白簡約、專業質感的網頁風格來設計此介面，謝謝！</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>請幫我製作一個 Windows 電腦上運行的原生桌面應用程式，用來監控 ASUS 官網的筆電價格，並在降價至期望價格以下時發送系統通知。請使用 Python 與 SQLite 開發，並以最簡潔、極致穩定的架構寫出完整程式碼，並告訴我如何執行。
+1. 系統架構與穩定性要求 (關鍵核心)
+- 行程分離設計：為避免 Playwright 瀏覽器自動化在非同步/多執行緒（如 Tkinter 背景執行緒或 pythonw.exe）下運行發生 Event Loop 死鎖或崩潰，必須將系統拆分為四個獨立的檔案：
+  1. database.py：負責 SQLite 資料庫 (price_monitor.db) 的初始化與所有增刪查改操作（包含警報規則、價格歷史與已發送通知紀錄）。資料庫路徑必須基於腳本的絕對路徑，以確保工作排程器執行時能正確定位。
+  2. scraper.py：獨立的爬蟲行程。由 main.py 透過 subprocess.run 啟動。使用 Playwright 無頭 Chromium 模擬滾動到底部以加載所有商品。爬取結果必須以 json.dumps(..., ensure_ascii=True) 序列化為 ASCII-escaped JSON 格式輸出至 stdout，過程日誌與錯誤則輸出至 stderr，以防止 Windows 控制台（如 CP950）在重導向 stdout 時因讀取到不相容字元而崩潰。
+  3. main.py：負責桌面 GUI 介面的展示與定時輪詢核心，支援獨立執行緒啟動 scraper.py，且支援 --headless 命令行參數。
+     - 隱藏執行：呼叫 scraper.py 時，若目前以 pythonw.exe 執行，必須自動替換為 python.exe（確保 Playwright 正常啟動），並透過設定 Windows startupinfo.wShowWindow = 0 (SW_HIDE) 旗標，將彈出的爬蟲 CMD 黑視窗完全隱藏。
+  4. run_app.bat：一鍵啟動批處理檔。用來雙擊直接執行 python main.py。若發生執行出錯，視窗應保持開啟並提示使用者安裝依賴（pip install customtkinter playwright）。
+- 無介面排程支援 (Headless Mode)：
+  main.py 必須支援 --headless 命令行參數（即執行 python main.py --headless）。在此模式下，程式不啟動 GUI 介面，而是直接在背景執行一次爬蟲調用、寫入資料庫、比對期望價規則、觸發系統通知後即自動關閉，以利配合 Windows 工作排程器定時執行。
+- 資料庫：在同目錄下使用 SQLite (price_monitor.db) 儲存規則、價格歷史，以及 notifications_sent 發送紀錄。
+2. 介面美感要求 (SaaS 科技藍雙色調儀表板)
+請使用 CustomTkinter (customtkinter) 庫進行扁平化現代設計（預設設為 AppearanceMode: light, ColorTheme: blue）：
+- 左側邊欄 (深色主題 - #0f172a)：
+  品牌名稱區、新增規則區、規則列表、監控開關與手動更新按鈕。
+  輸入框改為深色扁平設計 (fg_color="#1e293b", border_color="#334155")。由於 CTkEntry 不支援建構子內直接傳入 focused_border_color，必須手動綁定 &lt;FocusIn&gt; 與 &lt;FocusOut&gt; 事件，在 Focused 時將 border color 設為科技藍 #3b82f6 實現動態高亮。
+  規則列表的卡片使用 #1e293b 作為背景並包含紅色 × 的刪除按鈕。使用平面 Frame 與細線作為區塊分隔，不使用傳統的凹凸 LabelFrame 框。
+- 右側主面板 (淺色主題 - #f8fafc)：
+  頂部配置軟藍色 (#f1f5f9) 圓角膠囊狀態列，帶有綠色連線指示燈 ● （於自動更新/手動更新時變更顏色與文字狀態）與最後更新時間。
+  顯示兩個分頁：「目前最新價格」與「歷史更新紀錄」（以 CTkTabview 呈現）。
+- 響應式垂直卡片 (Latest Prices Tab)：
+  每台筆電為一個純白 (#ffffff) 懸浮卡片，具備灰色細框。透過遞迴綁定 &lt;Enter&gt; 與 &lt;Leave&gt; 事件（跳過 CTkButton），在滑鼠移入時將邊框顏色改為科技藍，移出時復原。
+  版面必須為垂直堆疊 (Vertical Stack)：上層為品名（Wraplength 設定為 700 左右，隨視窗縮小自動換行）；下層為左右對齊（左側為價格與漲跌幅度膠囊 Badge，右側為「查看歷史」按鈕）。這可確保縮小視窗時，按鈕與文字絕對不被遮擋或重疊。
+- 價格變化提示：比上次降價用綠色標章顯示 (↓ 降價金額，背景 #dcfce7，字體 #15803d)；漲價用紅色標章顯示 (↑ 漲價金額，背景 #fee2e2，字體 #b91c1c)；無變動用灰色顯示 (無變動)。
+- 斑馬紋數據表格 (Treeview)：
+  更新紀錄表格與單品歷史彈窗，使用標準 ttk.Treeview 並設定 style.theme_use('clam') 以便配置自訂色彩。將背景設為 #ffffff，奇數行設置標籤 odd 背景為 #f8fafc。配合使用 CTkScrollbar 替代傳統 Tkinter 滾動條以符合 CustomTkinter 設計語言，且移除 Treeview 預設的厚重外邊框。
+3. 功能細節要求
+- 爬蟲邏輯：爬取 https://www.asus.com/tw/laptops/for-home/all-series/filter?Spec=126640。啟動 Playwright 無頭 Chromium，模擬滾動到底部以加載所有商品（滾動 6 次，每次間隔 1.5 秒）。
+  - Selectors：商品卡片使用 div[class*="ProductCardNormalGrid__productCardContainer"]；商品名稱使用 a[class*="headingRow"] h2 或 a[class*="headingRow"]；連結使用 a[class*="headingRow"] 的 href 屬性；當前實售價使用 div[class*="ProductCardNormalGrid__price__"]（過濾掉含有 regularPrice 類名的刪除線原價）。
+- 警報通知：新增規則時，模糊比對商品品名（不區分大小寫）。當 當前實售價 &lt;= 期望價 時，若該商品在資料庫中為初次符合或價格有變動，調用 PowerShell BalloonTip 彈出 Windows 系統通知，不重複發送相同價格的通知。
+- 歷史彈窗與匯出：
+  點選卡片「查看歷史」彈出 CTkToplevel 模態小視窗，用表格列出此商品所有歷史價格。
+  支援「匯出全體歷史 (CSV)」與單品「下載歷史 (CSV)」。匯出 CSV 時，開啟檔案必須使用 Python 的 utf-8-sig 編碼寫入（即自動添加 UTF-8 BOM \ufeff 標記），以防止 Windows 使用者雙擊 Excel 直接開啟時中文內容產生亂碼。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Microsoft JhengHei UI"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>一</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>題：網站價格監控</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>第二題：信用卡記帳管理系統</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>第三題：PDF與圖片影像辨識匯入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>我手邊有一個記帳的 Excel 檔案「信用卡消費彙整表_題目.xlsm」，我希望能以這個檔案的資料和規則為基礎，幫我製作一個全新的網頁版記帳管理系統。
 請幫我完成以下所有步驟：
 1. 【分析與讀取 Excel】
@@ -1068,75 +1162,6 @@
      * 所有表格在手機上如果超出螢幕寬度，要能夠左右滑動檢視，不可以擠壓變形。
    - 請幫我寫一個 Windows 的一鍵啟動檔案（.bat），讓我雙擊就能直接啟動網頁並自動開啟瀏覽器。
 請以最乾淨、架構清晰的程式碼來實現這個系統，謝謝！</t>
-  </si>
-  <si>
-    <t>第二題：PDF與圖片影像辨識匯入</t>
-  </si>
-  <si>
-    <t>PDF解析是提取原生向量文字物件，並透過演算法進行結構重組；而圖片辨識則是藉由光學字元辨識(OCR)進行特徵提取與字元重建。</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>第三題：網站價格監控</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>利用 Playwright 進行自動網頁爬取，能定時監控網站商品的價格波動，並在售價低於期望值時自動提醒與匯出歷史報表。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>我想要在網頁上新增一個「批次檔案匯入」的功能，可以支援上傳信用卡對帳單的 PDF 檔或圖片檔（JPG, PNG），並自動抓取裡面的交易明細，具體需求如下：
-1. 檔案讀取方式：
-   - 如果是圖片檔，請利用離線 OCR 引擎（文字辨識）來辨識圖中的文字。
-   - 如果是 PDF 檔，因為裡面本來就有文字定義，請直接用 PDF 的文字提取方式讀取，不需要用 OCR，並請確保能把同一橫排的文字（日期、明細、金額）正確拼湊在一起，避免行與行之間對不齊。
-2. 資料抓取與雜訊過濾：
-   - 幫我從檔案內容中抓出每筆刷卡的：消費日期、消費明細（如果有英文字中間多餘的空格請幫我刪除）、消費金額、消費地區。
-   - 排除雜訊：帳單內常會出現「信用卡卡號、最低應繳金額、本期應繳總金額、結帳日、繳款截止日、持卡人姓名」等數字，請幫我寫規則過濾掉，不要把它們誤認成消費金額。
-3. 交易明細確認視窗（使用者審核介面）：
-   - 解析完成後，請彈出一個名為「交易明細確認」的簡約視窗，讓我們逐一確認每個檔案的內容：
-     - 視窗頂部要有一個「檔案審核進度條」（例如：第 1 / 3 個檔案），讓我知道還有幾張要確認。
-     - 頂部可以設定「此檔案所屬銀行」，並會自動偵測帳單文字來預填銀行名稱。
-     - 中間顯示一個簡約的 7 欄表格（刷卡日期、帳單起息日、明細、金額、地區、分類、操作），使用者可以直接在表格內手動修改，或者點操作欄的垃圾桶圖示刪除該筆錯誤資料。
-     - 視窗底部除了「取消」與「確認匯入資料庫」外，必須有「捨棄此檔案」按鈕，讓我可以跳過或刪除整張解析失敗的檔案。
-請以藍白簡約、專業質感的網頁風格來設計此介面，謝謝！</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>請幫我製作一個 Windows 電腦上運行的原生桌面應用程式，用來監控 ASUS 官網的筆電價格，並在降價至期望價格以下時發送系統通知。請使用 Python 與 SQLite 開發，並以最簡潔、極致穩定的架構寫出完整程式碼，並告訴我如何執行。
-1. 系統架構與穩定性要求 (關鍵核心)
-- 行程分離設計：為避免 Playwright 瀏覽器自動化在非同步/多執行緒（如 Tkinter 背景執行緒或 pythonw.exe）下運行發生 Event Loop 死鎖或崩潰，必須將系統拆分為四個獨立的檔案：
-  1. database.py：負責 SQLite 資料庫 (price_monitor.db) 的初始化與所有增刪查改操作（包含警報規則、價格歷史與已發送通知紀錄）。資料庫路徑必須基於腳本的絕對路徑，以確保工作排程器執行時能正確定位。
-  2. scraper.py：獨立的爬蟲行程。由 main.py 透過 subprocess.run 啟動。使用 Playwright 無頭 Chromium 模擬滾動到底部以加載所有商品。爬取結果必須以 json.dumps(..., ensure_ascii=True) 序列化為 ASCII-escaped JSON 格式輸出至 stdout，過程日誌與錯誤則輸出至 stderr，以防止 Windows 控制台（如 CP950）在重導向 stdout 時因讀取到不相容字元而崩潰。
-  3. main.py：負責桌面 GUI 介面的展示與定時輪詢核心，支援獨立執行緒啟動 scraper.py，且支援 --headless 命令行參數。
-     - 隱藏執行：呼叫 scraper.py 時，若目前以 pythonw.exe 執行，必須自動替換為 python.exe（確保 Playwright 正常啟動），並透過設定 Windows startupinfo.wShowWindow = 0 (SW_HIDE) 旗標，將彈出的爬蟲 CMD 黑視窗完全隱藏。
-  4. run_app.bat：一鍵啟動批處理檔。用來雙擊直接執行 python main.py。若發生執行出錯，視窗應保持開啟並提示使用者安裝依賴（pip install customtkinter playwright）。
-- 無介面排程支援 (Headless Mode)：
-  main.py 必須支援 --headless 命令行參數（即執行 python main.py --headless）。在此模式下，程式不啟動 GUI 介面，而是直接在背景執行一次爬蟲調用、寫入資料庫、比對期望價規則、觸發系統通知後即自動關閉，以利配合 Windows 工作排程器定時執行。
-- 資料庫：在同目錄下使用 SQLite (price_monitor.db) 儲存規則、價格歷史，以及 notifications_sent 發送紀錄。
-2. 介面美感要求 (SaaS 科技藍雙色調儀表板)
-請使用 CustomTkinter (customtkinter) 庫進行扁平化現代設計（預設設為 AppearanceMode: light, ColorTheme: blue）：
-- 左側邊欄 (深色主題 - #0f172a)：
-  品牌名稱區、新增規則區、規則列表、監控開關與手動更新按鈕。
-  輸入框改為深色扁平設計 (fg_color="#1e293b", border_color="#334155")。由於 CTkEntry 不支援建構子內直接傳入 focused_border_color，必須手動綁定 &lt;FocusIn&gt; 與 &lt;FocusOut&gt; 事件，在 Focused 時將 border color 設為科技藍 #3b82f6 實現動態高亮。
-  規則列表的卡片使用 #1e293b 作為背景並包含紅色 × 的刪除按鈕。使用平面 Frame 與細線作為區塊分隔，不使用傳統的凹凸 LabelFrame 框。
-- 右側主面板 (淺色主題 - #f8fafc)：
-  頂部配置軟藍色 (#f1f5f9) 圓角膠囊狀態列，帶有綠色連線指示燈 ● （於自動更新/手動更新時變更顏色與文字狀態）與最後更新時間。
-  顯示兩個分頁：「目前最新價格」與「歷史更新紀錄」（以 CTkTabview 呈現）。
-- 響應式垂直卡片 (Latest Prices Tab)：
-  每台筆電為一個純白 (#ffffff) 懸浮卡片，具備灰色細框。透過遞迴綁定 &lt;Enter&gt; 與 &lt;Leave&gt; 事件（跳過 CTkButton），在滑鼠移入時將邊框顏色改為科技藍，移出時復原。
-  版面必須為垂直堆疊 (Vertical Stack)：上層為品名（Wraplength 設定為 700 左右，隨視窗縮小自動換行）；下層為左右對齊（左側為價格與漲跌幅度膠囊 Badge，右側為「查看歷史」按鈕）。這可確保縮小視窗時，按鈕與文字絕對不被遮擋或重疊。
-- 價格變化提示：比上次降價用綠色標章顯示 (↓ 降價金額，背景 #dcfce7，字體 #15803d)；漲價用紅色標章顯示 (↑ 漲價金額，背景 #fee2e2，字體 #b91c1c)；無變動用灰色顯示 (無變動)。
-- 斑馬紋數據表格 (Treeview)：
-  更新紀錄表格與單品歷史彈窗，使用標準 ttk.Treeview 並設定 style.theme_use('clam') 以便配置自訂色彩。將背景設為 #ffffff，奇數行設置標籤 odd 背景為 #f8fafc。配合使用 CTkScrollbar 替代傳統 Tkinter 滾動條以符合 CustomTkinter 設計語言，且移除 Treeview 預設的厚重外邊框。
-3. 功能細節要求
-- 爬蟲邏輯：爬取 https://www.asus.com/tw/laptops/for-home/all-series/filter?Spec=126640。啟動 Playwright 無頭 Chromium，模擬滾動到底部以加載所有商品（滾動 6 次，每次間隔 1.5 秒）。
-  - Selectors：商品卡片使用 div[class*="ProductCardNormalGrid__productCardContainer"]；商品名稱使用 a[class*="headingRow"] h2 或 a[class*="headingRow"]；連結使用 a[class*="headingRow"] 的 href 屬性；當前實售價使用 div[class*="ProductCardNormalGrid__price__"]（過濾掉含有 regularPrice 類名的刪除線原價）。
-- 警報通知：新增規則時，模糊比對商品品名（不區分大小寫）。當 當前實售價 &lt;= 期望價 時，若該商品在資料庫中為初次符合或價格有變動，調用 PowerShell BalloonTip 彈出 Windows 系統通知，不重複發送相同價格的通知。
-- 歷史彈窗與匯出：
-  點選卡片「查看歷史」彈出 CTkToplevel 模態小視窗，用表格列出此商品所有歷史價格。
-  支援「匯出全體歷史 (CSV)」與單品「下載歷史 (CSV)」。匯出 CSV 時，開啟檔案必須使用 Python 的 utf-8-sig 編碼寫入（即自動添加 UTF-8 BOM \ufeff 標記），以防止 Windows 使用者雙擊 Excel 直接開啟時中文內容產生亂碼。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1144,7 +1169,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1180,6 +1205,13 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Microsoft JhengHei UI"/>
       <family val="2"/>
       <charset val="136"/>
     </font>
@@ -1239,7 +1271,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1257,6 +1289,12 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -1754,46 +1792,46 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" s="7" customFormat="1" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>46</v>
+      <c r="A18" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>